<commit_message>
besseres dashboard mit Guthaben display
</commit_message>
<xml_diff>
--- a/website/app/dashboard/components/Kostentabelle.xlsx
+++ b/website/app/dashboard/components/Kostentabelle.xlsx
@@ -1,20 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8BA11A-BF5A-4F57-BC69-B3987B4704F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Tabelle1" state="visible" r:id="rId4"/>
+    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>In game Name</t>
   </si>
@@ -25,6 +42,9 @@
     <t>.test</t>
   </si>
   <si>
+    <t>Javatest</t>
+  </si>
+  <si>
     <t xml:space="preserve">Passwort </t>
   </si>
   <si>
@@ -32,6 +52,9 @@
   </si>
   <si>
     <t>$2b$10$VMWECcA6bHFcEgP5YPz21e02weZ41DqNGxa7TnMwzfZHt8keZPppi</t>
+  </si>
+  <si>
+    <t>$2b$10$Mbmx0KfbHMWvv62pSIgDQuSZhz3OxuOc2Pn7XYZxdBOlzs3CMWRuG</t>
   </si>
   <si>
     <t>Geld eingezahlt</t>
@@ -64,33 +87,33 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00 &quot;€&quot;_-;-* #,##0.00 &quot;€&quot;_-;_-* &quot;-&quot;?? &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="[$-407]mmmm yy;@"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="[$-407]mmmm\ yy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="3">
@@ -126,12 +149,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -462,9 +485,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD34"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9.140625"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" customWidth="1"/>
@@ -474,7 +497,7 @@
     <col min="30" max="30" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,6 +506,9 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -501,67 +527,118 @@
       <c r="T1" s="1"/>
       <c r="AA1" s="2"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
       </c>
       <c r="AA2" s="2"/>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="4">
         <v>15</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4">
+        <v>0</v>
+      </c>
+      <c r="T3" s="4">
+        <v>0</v>
+      </c>
+      <c r="U3" s="4">
+        <v>0</v>
+      </c>
+      <c r="V3" s="4">
+        <v>0</v>
+      </c>
+      <c r="W3" s="4">
+        <v>0</v>
+      </c>
+      <c r="X3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="4">
+        <v>0</v>
+      </c>
       <c r="AA3" s="2"/>
       <c r="AB3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AC3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4">
-        <f>B3*0.2</f>
+        <f t="shared" ref="B4:Y4" si="0">IF(B3*0.2=0,0,B3*0.2)</f>
         <v>3</v>
       </c>
       <c r="C4" s="4">
-        <f t="shared" ref="C4:Z4" si="0">C3*0.2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D4" s="4">
@@ -653,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="Z4" s="4">
-        <f t="shared" si="0"/>
+        <f>IF(Z3*0.2=0,0,Z3*0.2)</f>
         <v>0</v>
       </c>
       <c r="AA4" s="2"/>
@@ -663,19 +740,19 @@
       </c>
       <c r="AC4" s="4">
         <f>AB4+SUM(AD8:AD33)</f>
-        <v>-200</v>
+        <v>-203.5</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4">
-        <f>B3-B4</f>
+        <f t="shared" ref="B5:Y5" si="1">IF(B3-B4=0,0,B3-B4)</f>
         <v>12</v>
       </c>
       <c r="C5" s="4">
-        <f t="shared" ref="C5:Z5" si="1">C3-C4</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="D5" s="4">
@@ -767,26 +844,26 @@
         <v>0</v>
       </c>
       <c r="Z5" s="4">
-        <f t="shared" si="1"/>
+        <f>IF(Z3-Z4=0,0,Z3-Z4)</f>
         <v>0</v>
       </c>
       <c r="AA5" s="2"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4">
-        <f>B5-0.5*COUNTIF(B8:B20,"WAHR")</f>
+        <f>IF(B5-0.5*COUNTIF(B8:B33,"WAHR")=0,0,(B5-0.5*COUNTIF(B8:B33,"WAHR")))</f>
         <v>10.5</v>
       </c>
       <c r="C6" s="4">
-        <f t="shared" ref="C6:Z6" si="2">C5-0.5*COUNTIF(C8:C20,"WAHR")</f>
+        <f>IF(C5-0.5*COUNTIF(C8:C33,"WAHR")=0,0,(C5-0.5*COUNTIF(C8:C33,"WAHR")))</f>
         <v>0</v>
       </c>
       <c r="D6" s="4">
-        <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <f t="shared" ref="D6:Z6" si="2">IF(D5-0.5*COUNTIF(D8:D33,"WAHR")=0,0,(D5-0.5*COUNTIF(D8:D33,"WAHR")))</f>
+        <v>0</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="2"/>
@@ -798,7 +875,7 @@
       </c>
       <c r="G6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
         <f t="shared" si="2"/>
@@ -818,7 +895,7 @@
       </c>
       <c r="L6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="M6" s="4">
         <f t="shared" si="2"/>
@@ -834,7 +911,7 @@
       </c>
       <c r="P6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="4">
         <f t="shared" si="2"/>
@@ -846,15 +923,15 @@
       </c>
       <c r="S6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="T6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="U6" s="4">
         <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="V6" s="4">
         <f t="shared" si="2"/>
@@ -880,7 +957,7 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -909,13 +986,13 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AC7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AD7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
@@ -926,10 +1003,10 @@
         <v>1</v>
       </c>
       <c r="C8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -938,7 +1015,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -953,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" t="b">
         <v>0</v>
@@ -965,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -974,13 +1051,13 @@
         <v>0</v>
       </c>
       <c r="S8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V8" t="b">
         <v>0</v>
@@ -1000,14 +1077,14 @@
       <c r="AA8" s="2"/>
       <c r="AB8" s="4">
         <f>0.5*COUNTIF($B8:Z8, "WAHR")</f>
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="AC8" s="4">
         <v>8</v>
       </c>
       <c r="AD8" s="4">
         <f>AB8-AC8</f>
-        <v>-4</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
@@ -3310,10 +3387,10 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>